<commit_message>
Add room photos with bookcase numbering; numbering is right-to-left
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VsNjZTxkuPm4Ex7K68Sd7T
</commit_message>
<xml_diff>
--- a/data/books-template.xlsx
+++ b/data/books-template.xlsx
@@ -232,7 +232,7 @@
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>لازم. رقم المكتبة بالغرفة (من جنب الباب مع عقارب الساعة).</t>
+        <t>لازم. رقم المكتبة بالغرفة، من اليمين لليسار (متل صور الترقيم).</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
@@ -54889,7 +54889,7 @@
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>٥. الترقيم: المكتبات من جنب الباب مع عقارب الساعة، والأقسام من اليمين، والرفوف من فوق.</t>
+          <t>٥. الترقيم: المكتبات والأقسام من اليمين لليسار (شوف صور الترقيم)، والرفوف من فوق.</t>
         </is>
       </c>
     </row>
@@ -54927,7 +54927,7 @@
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
         <is>
-          <t>• المكتبة: لازم. رقم المكتبة بالغرفة (من جنب الباب مع عقارب الساعة).</t>
+          <t>• المكتبة: لازم. رقم المكتبة بالغرفة، من اليمين لليسار (متل صور الترقيم).</t>
         </is>
       </c>
     </row>

</xml_diff>